<commit_message>
headless calls of the new GUI-inspired features
</commit_message>
<xml_diff>
--- a/monet/tests/TestData/control/power_database.xlsx
+++ b/monet/tests/TestData/control/power_database.xlsx
@@ -507,12 +507,12 @@
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>2022-07-25</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:23</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -533,12 +533,12 @@
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>2022-07-25</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:23</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -563,12 +563,12 @@
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>2022-07-25</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:23</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -589,12 +589,12 @@
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>2022-07-25</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:23</t>
         </is>
       </c>
       <c r="F5" t="n">

</xml_diff>